<commit_message>
chore: remove template code the system never runs
- trainer worker: the BERT/CoNLL training job from the project template and
  its dataset helpers are gone; the two retrain jobs share one wrapper and
  now record train_runs_total and train_duration_seconds themselves
- simple_worker.py (demo job) removed
- jobs API: POST /api/jobs and POST /api/jobs/train removed; the first put
  jobs on a queue no worker reads, the second queued the template job with
  arguments it did not accept. Queue inspection, status, cancel and retry stay
- scripts: test_all_endpoints.py (created accounts and buckets in the live
  system), verify_hatyai_api.py and seed_weather_history.py removed;
  api_snapshot regenerated from the running API (56 endpoints)
- frontend: four API wrappers without callers and their types removed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/api_snapshot.xlsx
+++ b/backend/scripts/api_snapshot.xlsx
@@ -426,13 +426,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="53" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="35" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
   </cols>
@@ -673,18 +673,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/api/storage/buckets</t>
+          <t>/api/stations</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>List Buckets</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr"/>
+          <t>List Active Solar Stations</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ดึงรายชื่อสถานีโซลาร์ฟาร์มทั้งหมด พร้อมข้อมูลกำลังผลิตจริงจากฐานข้อมูล</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -701,18 +705,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/api/storage/buckets</t>
+          <t>/api/stations</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Create Bucket</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr"/>
+          <t>Create New Solar Station</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ลงทะเบียนสถานีโรงไฟฟ้าโซลาร์แห่งใหม่</t>
+        </is>
+      </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -724,23 +732,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/api/storage/upload</t>
+          <t>/api/stations/archived</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Upload File</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr"/>
+          <t>List Archived / Soft-Deleted Stations</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ดึงรายชื่อสถานีที่ถูกระงับการใช้งาน (Soft-deleted) ทั้งหมด</t>
+        </is>
+      </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -757,18 +769,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/api/storage/download/{bucket_name}/{object_name}</t>
+          <t>/api/stations/nearest</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Download File</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr"/>
+          <t>Find Nearest Solar Station by Coordinates</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ค้นหาสถานีโซลาร์ฟาร์มที่อยู่ใกล้พิกัด Latitude/Longitude มากที่สุด (Nearest Mapping)</t>
+        </is>
+      </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -780,23 +796,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>PUT</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/api/storage/buckets/{bucket_name}/versioning</t>
+          <t>/api/stations/{station_id}</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Set Versioning</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr"/>
+          <t>Get Station Detail by ID</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>ดึงข้อมูลรายละเอียดและสเปกของสถานีตาม ID พร้อมค่ากำลังผลิตล่าสุด</t>
+        </is>
+      </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>storage</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -808,23 +828,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>PUT</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/api/label-studio/projects</t>
+          <t>/api/stations/{station_id}</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>List Projects</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
+          <t>Full Update Station Spec</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>อัปเดตข้อมูลสเปกของสถานีทั้งหมด (Full Update)</t>
+        </is>
+      </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>label-studio</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -836,23 +860,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/api/label-studio/projects</t>
+          <t>/api/stations/{station_id}</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Create Project</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>Partial Update Station Spec</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>แก้ไขเฉพาะบางฟิลด์ของสถานี (Partial Update)</t>
+        </is>
+      </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>label-studio</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -864,23 +892,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/api/label-studio/projects/{project_id}/tasks</t>
+          <t>/api/stations/{station_id}</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>List Tasks</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr"/>
+          <t>Soft-Delete / Deactivate Station</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>ปิดการใช้งานสถานีชั่วคราว (Soft-Delete) โดยไม่ลบประวัติใน DB</t>
+        </is>
+      </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>label-studio</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -892,23 +924,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>PATCH</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>/api/label-studio/projects/{project_id}/tasks</t>
+          <t>/api/stations/{station_id}/restore</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Create Task</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr"/>
+          <t>Restore Soft-Deleted Station</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>กู้คืนสถานีที่เคยถูกระงับการใช้งานกลับมาทำงานใหม่ (Restore)</t>
+        </is>
+      </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>label-studio</t>
+          <t>stations</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -920,23 +956,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>/api/jobs/</t>
+          <t>/api/dashboard/summary</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Enqueue Job</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
+          <t>System-wide Dashboard Overview (KPI Cards)</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>สรุปภาพรวมทั้งระบบขึ้นหน้าแรก (KPI Cards, กำลังผลิตรวม, ความเสี่ยงรวม)</t>
+        </is>
+      </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>jobs</t>
+          <t>dashboard</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -953,18 +993,22 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>/api/jobs/{job_id}</t>
+          <t>/api/dashboard/alerts</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Get Job Status</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr"/>
+          <t>Real-time Alert Feeds for Critical / Warning Stations</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>ดึงรายการแจ้งเตือนด่วน (Real-time Alert Feeds) ที่ต้องการเฝ้าระวังหรือเร่งสำรองไฟ</t>
+        </is>
+      </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>jobs</t>
+          <t>dashboard</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -981,25 +1025,1161 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>/api/dashboard/grafana-links</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Get Observability Grafana Dashboard Links</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ดึง URL สำหรับ Embed หรือเปิดดู Grafana Dashboards</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>dashboard</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>/api/dashboard/station/{station_id}</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Station-Specific Dashboard Detail (Forecast Curve + Cloud Trend)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ดึงข้อมูลแดชบอร์ดเฉพาะสถานี (กราฟพยากรณ์ 3 ชม., ทัศนวิสัยเมฆ, คำแนะนำ ΔP)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>dashboard</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>/api/storage/buckets</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>List Buckets</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>/api/storage/buckets</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Create Bucket</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>/api/storage/upload</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Upload File</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>/api/storage/download/{bucket_name}/{object_name}</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Download File</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>PUT</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>/api/storage/buckets/{bucket_name}/versioning</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Set Versioning</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>/api/label-studio/projects</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>List Projects</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>/api/label-studio/projects</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Create Project</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>/api/label-studio/projects/{project_id}/tasks</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>List Tasks</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>/api/label-studio/projects/{project_id}/tasks</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Create Task</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>/api/label-studio/projects/{project_id}/tasks/{task_id}/annotations</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>List Annotations</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>/api/label-studio/projects/{project_id}/tasks/{task_id}/annotations</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Create Annotation</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>/api/label-studio/ground-truth/submit</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Submit Ground Truth</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>ส่ง GHI จริง 1 ค่า -&gt; Label Studio (สร้าง/อัปเดต) -&gt; นัด retrain.</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>/api/label-studio/ground-truth/batch-submit</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Batch Submit Ground Truth</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>ส่ง GHI จริงหลายค่า (จากตารางหน้าเว็บ).</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>/api/label-studio/ground-truth/upload/preview</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Preview Ground Truth File</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>อ่านหัวตาราง + ตัวอย่างแถวของไฟล์ และเดาคอลัมน์เวลา/GHI ให้ผู้ใช้เลือกยืนยัน.</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>/api/label-studio/ground-truth/upload</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Upload Ground Truth File</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>นำเข้า GHI จริงจากไฟล์ CSV/XLSX เฉพาะแถวที่อยู่ในวันที่เลือก (เวลาไทย) ตามคอลัมน์ที่ผู้ใช้ระบุ.</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>label-studio</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>/api/jobs/queues</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Summary of All Redis Task Queues</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>สรุปภาพรวมของทุกคิวใน Redis (จำนวนงานที่รอ, กำลังรัน, พัง)</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>/api/jobs/queues/{name}/jobs</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>List Pending Jobs in a Specific Queue</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>ดูรายการ Job ทั้งหมดที่ค้างอยู่ในคิวที่เลือก</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>/api/jobs/queues/{name}/clear</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Clear / Flush All Pending Jobs in a Queue</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>ล้างคิวงานทั้งหมด (Flush Pending Jobs)</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>/api/jobs/{job_id}/retry</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Retry a Failed Job</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>สั่งให้ Job ที่เคย Failed รันใหม่อีกครั้ง</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>/api/jobs/{job_id}</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Get Job Status and Result</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>DELETE</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>/api/jobs/{job_id}</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Cancel / Remove Job from Queue</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>ยกเลิก / ลบ Job ออกจากคิวทันท่วงที (Cancel Job)</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>/api/inference/predict</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Enqueue 3-Hour Solar Forecast Request</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>สั่งคำขอพยากรณ์ไฟฟ้าล่วงหน้า 3 ชม. (Enqueue to inference_queue)</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>inference</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>/api/inference/result/{job_id}</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Get Forecast Result by Job ID</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>ดึงผลลัพธ์การพยากรณ์เมื่อ Worker ประมวลผลเสร็จ</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>inference</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>/api/inference/latest/{station_id}</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Get Latest Pre-computed Forecast for Station Dashboard</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ดึงผลการพยากรณ์รอบล่าสุดของสถานีขึ้นแสดงบน Dashboard ทันที</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>inference</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>/api/inference/history/{station_id}</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Get Historical Forecasts for Comparison</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>ดึงประวัติผลพยากรณ์ย้อนหลังเพื่อนำไปพลอตกราฟเปรียบเทียบ</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>inference</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>/api/inference/predictions-by-date</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Forecasts of a day aligned to real time, with ground-truth labels</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ค่าพยากรณ์ + GHI จาก weather_history ของวันที่เลือก (เรียงตามเวลาจริง) + ค่าจริงที่ label ไว้แล้ว สำหรับหน้า labeling.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>inference</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>/api/ingestion/trigger</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Trigger Real-time Weather &amp; Satellite Ingestion</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>สั่งดึงข้อมูลสภาพอากาศแบบ Real-time (Open-Meteo) และภาพดาวเทียม Himawari (NICT) เข้าสู่ระบบทันที</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>ingestion</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>/api/ingestion/catchup</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Trigger Auto Catch-up / Gap Backfill for Station</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>สั่งตรวจสอบ Gap ของข้อมูลและดึงข้อมูลย้อนหลังทั้ง Weather Time-Series และภาพถ่ายดาวเทียม 12 เฟรมอัตโนมัติ</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>ingestion</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>/api/ingestion/weather/{station_id}/recent</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Get Normalized Weather Time-series for Station</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ดึงข้อมูลสภาพอากาศย้อนหลังระดับ Canonical Schema เพื่อใช้เป็น Input สำหรับโมเดล LSTM</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>ingestion</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>/api/ingestion/satellite/{station_id}/frames</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Get Recent Satellite Frame Sequences</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ดึงประวัติ URL ภาพถ่ายดาวเทียม Himawari ล่าสุดเพื่อใช้ส่งให้ ConvLSTM Cloud Motion Model</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>ingestion</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>/api/ingestion/status</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Get Ingestion Health &amp; Metrics</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ตรวจสอบสถานะสุขภาพและการเชื่อมต่อ Data Source (Open-Meteo, NICT Himawari) และจำนวนข้อมูลในระบบ</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>ingestion</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>/api/ingestion/satellite/{station_id}/latest.png</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Newest real satellite crop around a station (PNG)</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ภาพดาวเทียมจริงล่าสุดรอบสถานี (true-colour 64x64 พิกเซล) ที่ inference worker เก็บไว้ใน MinIO.</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>ingestion</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>/api/frame-review/frames</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>List Frames</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Real daytime satellite frames of one station and day, with automatic hints and the saved reviews.</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>frame-review</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>/api/frame-review/frames</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Submit Reviews</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Save the reviewer's verdicts. Rejected frames are left out of the next ConvLSTM retrain.</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>frame-review</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>/api/frame-review/status</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Convlstm Status</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Batch counter of new satellite scans, the deployed ConvLSTM and the result of the last retrain.</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>frame-review</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
           <t>/health</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C57" t="inlineStr">
         <is>
           <t>Health Check</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D57" t="inlineStr">
         <is>
           <t>ตรวจสอบว่า API server ทำงานปกติ</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E57" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F57" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
docs: day view, cloud player, inputs and retrain pages; results of 5 Oct evening
- README: check of the satellite relation at ST-003, error by lead time for
  the afternoon of 5 Oct (the blend helps at 10 minutes, not at 60-120),
  the automatic ConvLSTM retrain and the LSTM run with ST-003 labels, the
  pages that show a whole day, the in-memory copy of the labels, and three
  known limits (wind unit and DHI of the LSTM input, the two-hour gap after
  one missing frame)
- PLAN: status rows for the evening's work, limits updated
- backend, service and frontend READMEs: new endpoints, pages and the stored
  forecast frames; api_snapshot regenerated (58 endpoints)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/api_snapshot.xlsx
+++ b/backend/scripts/api_snapshot.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F57"/>
+  <dimension ref="A1:F59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1851,7 +1851,8 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>ค่าพยากรณ์ + GHI จาก weather_history ของวันที่เลือก (เรียงตามเวลาจริง) + ค่าจริงที่ label ไว้แล้ว สำหรับหน้า labeling.</t>
+          <t>ค่าพยากรณ์ + GHI จาก weather_history ของวันที่เลือก (เรียงตามเวลาจริง) + ค่าจริงที่ label ไว้แล้ว
+ใช้ทั้งหน้า labeling (predicted_ghi = รอบล่าสุด) และกราฟทั้งวันของหน้าพยากรณ์ (forecast_* ตาม lead_minutes).</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -2065,22 +2066,22 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/api/frame-review/frames</t>
+          <t>/api/ingestion/satellite/{station_id}/day-frames</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>List Frames</t>
+          <t>Real satellite frames of a day and the newest ConvLSTM forecast frames</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Real daytime satellite frames of one station and day, with automatic hints and the saved reviews.</t>
+          <t>Real Band 03 frames of one station and day, and for today the frames the ConvLSTM predicted in the newest round.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>frame-review</t>
+          <t>ingestion</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
@@ -2092,7 +2093,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2102,12 +2103,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Submit Reviews</t>
+          <t>List Frames</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Save the reviewer's verdicts. Rejected frames are left out of the next ConvLSTM retrain.</t>
+          <t>Real daytime satellite frames of one station and day, with automatic hints and the saved reviews.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -2124,22 +2125,22 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>/api/frame-review/status</t>
+          <t>/api/frame-review/frames</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Convlstm Status</t>
+          <t>Submit Reviews</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Batch counter of new satellite scans, the deployed ConvLSTM and the result of the last retrain.</t>
+          <t>Save the reviewer's verdicts. Rejected frames are left out of the next ConvLSTM retrain.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2161,25 +2162,89 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
+          <t>/api/frame-review/status</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Convlstm Status</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Batch counter of new satellite scans, the deployed ConvLSTM and the result of the last retrain.</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>frame-review</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>/api/retrain/status</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Deployed models, pending retrains and the retrain history of both models</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Deployed versions, what is pending and the retrain history of the LSTM and the ConvLSTM.</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>retrain</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
           <t>/health</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Health Check</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>ตรวจสอบว่า API server ทำงานปกติ</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F59" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
docs: automatic calibration check, learning curves, dark theme, course topics used
- README: how a station gets checked now, the learning curves and where they
  are stored, the dark theme, and a table of which course topics (241-353
  slides) the system uses and which it does not
- PLAN: status rows for the three additions
- backend, service and frontend READMEs: new endpoints, the trainer's third
  job, curves.py, and how to keep the two themes in step
- api_snapshot regenerated (60 endpoints)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/api_snapshot.xlsx
+++ b/backend/scripts/api_snapshot.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F59"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1392,22 +1392,22 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>/api/label-studio/ground-truth/submit</t>
+          <t>/api/label-studio/ground-truth/calibration-status</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Submit Ground Truth</t>
+          <t>Has the satellite relation been compared with measured GHI of this station?</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>ส่ง GHI จริง 1 ค่า -&gt; Label Studio (สร้าง/อัปเดต) -&gt; นัด retrain.</t>
+          <t>สูตรแสงจากภาพดาวเทียมเทียบกับค่าวัดจริงของสถานีนี้แล้วหรือยัง (ผลของงาน check_satellite_calibration ที่รันเองหลังบันทึกค่าวัดจริง).</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -1429,17 +1429,17 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>/api/label-studio/ground-truth/batch-submit</t>
+          <t>/api/label-studio/ground-truth/submit</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Batch Submit Ground Truth</t>
+          <t>Submit Ground Truth</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>ส่ง GHI จริงหลายค่า (จากตารางหน้าเว็บ).</t>
+          <t>ส่ง GHI จริง 1 ค่า -&gt; Label Studio (สร้าง/อัปเดต) -&gt; นัด retrain.</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -1461,17 +1461,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>/api/label-studio/ground-truth/upload/preview</t>
+          <t>/api/label-studio/ground-truth/batch-submit</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Preview Ground Truth File</t>
+          <t>Batch Submit Ground Truth</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>อ่านหัวตาราง + ตัวอย่างแถวของไฟล์ และเดาคอลัมน์เวลา/GHI ให้ผู้ใช้เลือกยืนยัน.</t>
+          <t>ส่ง GHI จริงหลายค่า (จากตารางหน้าเว็บ).</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1493,17 +1493,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>/api/label-studio/ground-truth/upload</t>
+          <t>/api/label-studio/ground-truth/upload/preview</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Upload Ground Truth File</t>
+          <t>Preview Ground Truth File</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>นำเข้า GHI จริงจากไฟล์ CSV/XLSX เฉพาะแถวที่อยู่ในวันที่เลือก (เวลาไทย) ตามคอลัมน์ที่ผู้ใช้ระบุ.</t>
+          <t>อ่านหัวตาราง + ตัวอย่างแถวของไฟล์ และเดาคอลัมน์เวลา/GHI ให้ผู้ใช้เลือกยืนยัน.</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1520,27 +1520,27 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>/api/jobs/queues</t>
+          <t>/api/label-studio/ground-truth/upload</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Summary of All Redis Task Queues</t>
+          <t>Upload Ground Truth File</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>สรุปภาพรวมของทุกคิวใน Redis (จำนวนงานที่รอ, กำลังรัน, พัง)</t>
+          <t>นำเข้า GHI จริงจากไฟล์ CSV/XLSX เฉพาะแถวที่อยู่ในวันที่เลือก (เวลาไทย) ตามคอลัมน์ที่ผู้ใช้ระบุ.</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>jobs</t>
+          <t>label-studio</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1557,17 +1557,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>/api/jobs/queues/{name}/jobs</t>
+          <t>/api/jobs/queues</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>List Pending Jobs in a Specific Queue</t>
+          <t>Summary of All Redis Task Queues</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>ดูรายการ Job ทั้งหมดที่ค้างอยู่ในคิวที่เลือก</t>
+          <t>สรุปภาพรวมของทุกคิวใน Redis (จำนวนงานที่รอ, กำลังรัน, พัง)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1584,22 +1584,22 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>/api/jobs/queues/{name}/clear</t>
+          <t>/api/jobs/queues/{name}/jobs</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Clear / Flush All Pending Jobs in a Queue</t>
+          <t>List Pending Jobs in a Specific Queue</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>ล้างคิวงานทั้งหมด (Flush Pending Jobs)</t>
+          <t>ดูรายการ Job ทั้งหมดที่ค้างอยู่ในคิวที่เลือก</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1616,22 +1616,22 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>/api/jobs/{job_id}/retry</t>
+          <t>/api/jobs/queues/{name}/clear</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Retry a Failed Job</t>
+          <t>Clear / Flush All Pending Jobs in a Queue</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>สั่งให้ Job ที่เคย Failed รันใหม่อีกครั้ง</t>
+          <t>ล้างคิวงานทั้งหมด (Flush Pending Jobs)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1648,20 +1648,24 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>/api/jobs/{job_id}</t>
+          <t>/api/jobs/{job_id}/retry</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Get Job Status and Result</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>Retry a Failed Job</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>สั่งให้ Job ที่เคย Failed รันใหม่อีกครั้ง</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
           <t>jobs</t>
@@ -1676,7 +1680,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DELETE</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1686,14 +1690,10 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Cancel / Remove Job from Queue</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>ยกเลิก / ลบ Job ออกจากคิวทันท่วงที (Cancel Job)</t>
-        </is>
-      </c>
+          <t>Get Job Status and Result</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
           <t>jobs</t>
@@ -1708,27 +1708,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>DELETE</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>/api/inference/predict</t>
+          <t>/api/jobs/{job_id}</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Enqueue 3-Hour Solar Forecast Request</t>
+          <t>Cancel / Remove Job from Queue</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>สั่งคำขอพยากรณ์ไฟฟ้าล่วงหน้า 3 ชม. (Enqueue to inference_queue)</t>
+          <t>ยกเลิก / ลบ Job ออกจากคิวทันท่วงที (Cancel Job)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>inference</t>
+          <t>jobs</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -1740,22 +1740,22 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>/api/inference/result/{job_id}</t>
+          <t>/api/inference/predict</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Get Forecast Result by Job ID</t>
+          <t>Enqueue 3-Hour Solar Forecast Request</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>ดึงผลลัพธ์การพยากรณ์เมื่อ Worker ประมวลผลเสร็จ</t>
+          <t>สั่งคำขอพยากรณ์ไฟฟ้าล่วงหน้า 3 ชม. (Enqueue to inference_queue)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1777,17 +1777,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>/api/inference/latest/{station_id}</t>
+          <t>/api/inference/result/{job_id}</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Get Latest Pre-computed Forecast for Station Dashboard</t>
+          <t>Get Forecast Result by Job ID</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>ดึงผลการพยากรณ์รอบล่าสุดของสถานีขึ้นแสดงบน Dashboard ทันที</t>
+          <t>ดึงผลลัพธ์การพยากรณ์เมื่อ Worker ประมวลผลเสร็จ</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1809,17 +1809,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>/api/inference/history/{station_id}</t>
+          <t>/api/inference/latest/{station_id}</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Get Historical Forecasts for Comparison</t>
+          <t>Get Latest Pre-computed Forecast for Station Dashboard</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>ดึงประวัติผลพยากรณ์ย้อนหลังเพื่อนำไปพลอตกราฟเปรียบเทียบ</t>
+          <t>ดึงผลการพยากรณ์รอบล่าสุดของสถานีขึ้นแสดงบน Dashboard ทันที</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1841,55 +1841,55 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>/api/inference/history/{station_id}</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Get Historical Forecasts for Comparison</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>ดึงประวัติผลพยากรณ์ย้อนหลังเพื่อนำไปพลอตกราฟเปรียบเทียบ</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>inference</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>/api/inference/predictions-by-date</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
         <is>
           <t>Forecasts of a day aligned to real time, with ground-truth labels</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D48" t="inlineStr">
         <is>
           <t>ค่าพยากรณ์ + GHI จาก weather_history ของวันที่เลือก (เรียงตามเวลาจริง) + ค่าจริงที่ label ไว้แล้ว
 ใช้ทั้งหน้า labeling (predicted_ghi = รอบล่าสุด) และกราฟทั้งวันของหน้าพยากรณ์ (forecast_* ตาม lead_minutes).</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E48" t="inlineStr">
         <is>
           <t>inference</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>POST</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>/api/ingestion/trigger</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>Trigger Real-time Weather &amp; Satellite Ingestion</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>สั่งดึงข้อมูลสภาพอากาศแบบ Real-time (Open-Meteo) และภาพดาวเทียม Himawari (NICT) เข้าสู่ระบบทันที</t>
-        </is>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>ingestion</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
@@ -1906,17 +1906,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/api/ingestion/catchup</t>
+          <t>/api/ingestion/trigger</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Trigger Auto Catch-up / Gap Backfill for Station</t>
+          <t>Trigger Real-time Weather &amp; Satellite Ingestion</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>สั่งตรวจสอบ Gap ของข้อมูลและดึงข้อมูลย้อนหลังทั้ง Weather Time-Series และภาพถ่ายดาวเทียม 12 เฟรมอัตโนมัติ</t>
+          <t>สั่งดึงข้อมูลสภาพอากาศแบบ Real-time (Open-Meteo) และภาพดาวเทียม Himawari (NICT) เข้าสู่ระบบทันที</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1933,22 +1933,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/api/ingestion/weather/{station_id}/recent</t>
+          <t>/api/ingestion/catchup</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Get Normalized Weather Time-series for Station</t>
+          <t>Trigger Auto Catch-up / Gap Backfill for Station</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>ดึงข้อมูลสภาพอากาศย้อนหลังระดับ Canonical Schema เพื่อใช้เป็น Input สำหรับโมเดล LSTM</t>
+          <t>สั่งตรวจสอบ Gap ของข้อมูลและดึงข้อมูลย้อนหลังทั้ง Weather Time-Series และภาพถ่ายดาวเทียม 12 เฟรมอัตโนมัติ</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1970,17 +1970,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>/api/ingestion/satellite/{station_id}/frames</t>
+          <t>/api/ingestion/weather/{station_id}/recent</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Get Recent Satellite Frame Sequences</t>
+          <t>Get Normalized Weather Time-series for Station</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ดึงประวัติ URL ภาพถ่ายดาวเทียม Himawari ล่าสุดเพื่อใช้ส่งให้ ConvLSTM Cloud Motion Model</t>
+          <t>ดึงข้อมูลสภาพอากาศย้อนหลังระดับ Canonical Schema เพื่อใช้เป็น Input สำหรับโมเดล LSTM</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2002,17 +2002,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>/api/ingestion/status</t>
+          <t>/api/ingestion/satellite/{station_id}/frames</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Get Ingestion Health &amp; Metrics</t>
+          <t>Get Recent Satellite Frame Sequences</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ตรวจสอบสถานะสุขภาพและการเชื่อมต่อ Data Source (Open-Meteo, NICT Himawari) และจำนวนข้อมูลในระบบ</t>
+          <t>ดึงประวัติ URL ภาพถ่ายดาวเทียม Himawari ล่าสุดเพื่อใช้ส่งให้ ConvLSTM Cloud Motion Model</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2034,17 +2034,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>/api/ingestion/satellite/{station_id}/latest.png</t>
+          <t>/api/ingestion/status</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Newest real satellite crop around a station (PNG)</t>
+          <t>Get Ingestion Health &amp; Metrics</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ภาพดาวเทียมจริงล่าสุดรอบสถานี (true-colour 64x64 พิกเซล) ที่ inference worker เก็บไว้ใน MinIO.</t>
+          <t>ตรวจสอบสถานะสุขภาพและการเชื่อมต่อ Data Source (Open-Meteo, NICT Himawari) และจำนวนข้อมูลในระบบ</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2066,17 +2066,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/api/ingestion/satellite/{station_id}/day-frames</t>
+          <t>/api/ingestion/satellite/{station_id}/latest.png</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Real satellite frames of a day and the newest ConvLSTM forecast frames</t>
+          <t>Newest real satellite crop around a station (PNG)</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Real Band 03 frames of one station and day, and for today the frames the ConvLSTM predicted in the newest round.</t>
+          <t>ภาพดาวเทียมจริงล่าสุดรอบสถานี (true-colour 64x64 พิกเซล) ที่ inference worker เก็บไว้ใน MinIO.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2098,22 +2098,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>/api/frame-review/frames</t>
+          <t>/api/ingestion/satellite/{station_id}/day-frames</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>List Frames</t>
+          <t>Real satellite frames of a day and the newest ConvLSTM forecast frames</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Real daytime satellite frames of one station and day, with automatic hints and the saved reviews.</t>
+          <t>Real Band 03 frames of one station and day, and for today the frames the ConvLSTM predicted in the newest round.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>frame-review</t>
+          <t>ingestion</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2125,7 +2125,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2135,12 +2135,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Submit Reviews</t>
+          <t>List Frames</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Save the reviewer's verdicts. Rejected frames are left out of the next ConvLSTM retrain.</t>
+          <t>Real daytime satellite frames of one station and day, with automatic hints and the saved reviews.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2157,22 +2157,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>/api/frame-review/status</t>
+          <t>/api/frame-review/frames</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Convlstm Status</t>
+          <t>Submit Reviews</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Batch counter of new satellite scans, the deployed ConvLSTM and the result of the last retrain.</t>
+          <t>Save the reviewer's verdicts. Rejected frames are left out of the next ConvLSTM retrain.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2194,22 +2194,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>/api/retrain/status</t>
+          <t>/api/frame-review/status</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Deployed models, pending retrains and the retrain history of both models</t>
+          <t>Convlstm Status</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Deployed versions, what is pending and the retrain history of the LSTM and the ConvLSTM.</t>
+          <t>Batch counter of new satellite scans, the deployed ConvLSTM and the result of the last retrain.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>retrain</t>
+          <t>frame-review</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2226,25 +2226,89 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
+          <t>/api/retrain/status</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Deployed models, pending retrains and the retrain history of both models</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Deployed versions, what is pending and the retrain history of the LSTM and the ConvLSTM.</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>retrain</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>/api/retrain/runs/{run_id}/curves</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Per-epoch learning curves of one retrain run</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Learning curves of one retrain run: training loss, validation metric and learning rate per epoch.</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>retrain</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>GET</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
           <t>/health</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C61" t="inlineStr">
         <is>
           <t>Health Check</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>ตรวจสอบว่า API server ทำงานปกติ</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>system</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F61" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
chore: remove the manual ingestion trigger; cleanup script lists the rows older versions left behind
POST /api/ingestion/trigger always answered "completed", stored the full-disk
image in place of the station's B03 crop when that crop was not there yet, and
did not check for rows already stored. No page or job called it, so it is
removed with the worker job ingest_single_station and the three image fetchers
only it used. POST /api/ingestion/catchup remains for a manual pull.

cleanup_test_data.py gets a section "leftovers": frame rows that point at the
full-disk image, exact copies of weather rows, and the full-disk files. It
lists them and deletes only with --apply and a typed confirmation.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/api_snapshot.xlsx
+++ b/backend/scripts/api_snapshot.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1906,17 +1906,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>/api/ingestion/trigger</t>
+          <t>/api/ingestion/catchup</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Trigger Real-time Weather &amp; Satellite Ingestion</t>
+          <t>Trigger Auto Catch-up / Gap Backfill for Station</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>สั่งดึงข้อมูลสภาพอากาศแบบ Real-time (Open-Meteo) และภาพดาวเทียม Himawari (NICT) เข้าสู่ระบบทันที</t>
+          <t>สั่งตรวจสอบ Gap ของข้อมูลและดึงข้อมูลย้อนหลังทั้ง Weather Time-Series และภาพถ่ายดาวเทียม 12 เฟรมอัตโนมัติ</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1933,22 +1933,22 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>/api/ingestion/catchup</t>
+          <t>/api/ingestion/weather/{station_id}/recent</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Trigger Auto Catch-up / Gap Backfill for Station</t>
+          <t>Get Normalized Weather Time-series for Station</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>สั่งตรวจสอบ Gap ของข้อมูลและดึงข้อมูลย้อนหลังทั้ง Weather Time-Series และภาพถ่ายดาวเทียม 12 เฟรมอัตโนมัติ</t>
+          <t>ดึงข้อมูลสภาพอากาศย้อนหลังระดับ Canonical Schema เพื่อใช้เป็น Input สำหรับโมเดล LSTM</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -1970,17 +1970,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>/api/ingestion/weather/{station_id}/recent</t>
+          <t>/api/ingestion/satellite/{station_id}/frames</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Get Normalized Weather Time-series for Station</t>
+          <t>Get Recent Satellite Frame Sequences</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>ดึงข้อมูลสภาพอากาศย้อนหลังระดับ Canonical Schema เพื่อใช้เป็น Input สำหรับโมเดล LSTM</t>
+          <t>ดึงประวัติ URL ภาพถ่ายดาวเทียม Himawari ล่าสุดเพื่อใช้ส่งให้ ConvLSTM Cloud Motion Model</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -2002,17 +2002,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>/api/ingestion/satellite/{station_id}/frames</t>
+          <t>/api/ingestion/status</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Get Recent Satellite Frame Sequences</t>
+          <t>Get Ingestion Health &amp; Metrics</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>ดึงประวัติ URL ภาพถ่ายดาวเทียม Himawari ล่าสุดเพื่อใช้ส่งให้ ConvLSTM Cloud Motion Model</t>
+          <t>ตรวจสอบสถานะสุขภาพและการเชื่อมต่อ Data Source (Open-Meteo, NICT Himawari) และจำนวนข้อมูลในระบบ</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -2034,17 +2034,17 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>/api/ingestion/status</t>
+          <t>/api/ingestion/satellite/{station_id}/latest.png</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Get Ingestion Health &amp; Metrics</t>
+          <t>Newest real satellite crop around a station (PNG)</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>ตรวจสอบสถานะสุขภาพและการเชื่อมต่อ Data Source (Open-Meteo, NICT Himawari) และจำนวนข้อมูลในระบบ</t>
+          <t>ภาพดาวเทียมจริงล่าสุดรอบสถานี (true-colour 64x64 พิกเซล) ที่ inference worker เก็บไว้ใน MinIO.</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -2066,17 +2066,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>/api/ingestion/satellite/{station_id}/latest.png</t>
+          <t>/api/ingestion/satellite/{station_id}/day-frames</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Newest real satellite crop around a station (PNG)</t>
+          <t>Real satellite frames of a day and the newest ConvLSTM forecast frames</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>ภาพดาวเทียมจริงล่าสุดรอบสถานี (true-colour 64x64 พิกเซล) ที่ inference worker เก็บไว้ใน MinIO.</t>
+          <t>Real Band 03 frames of one station and day, and for today the frames the ConvLSTM predicted in the newest round.</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -2098,22 +2098,22 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>/api/ingestion/satellite/{station_id}/day-frames</t>
+          <t>/api/frame-review/frames</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Real satellite frames of a day and the newest ConvLSTM forecast frames</t>
+          <t>List Frames</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Real Band 03 frames of one station and day, and for today the frames the ConvLSTM predicted in the newest round.</t>
+          <t>Real daytime satellite frames of one station and day, with automatic hints and the saved reviews.</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>ingestion</t>
+          <t>frame-review</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -2125,7 +2125,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>GET</t>
+          <t>POST</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2135,12 +2135,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>List Frames</t>
+          <t>Submit Reviews</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Real daytime satellite frames of one station and day, with automatic hints and the saved reviews.</t>
+          <t>Save the reviewer's verdicts. Rejected frames are left out of the next ConvLSTM retrain.</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -2157,22 +2157,22 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>POST</t>
+          <t>GET</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>/api/frame-review/frames</t>
+          <t>/api/frame-review/status</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Submit Reviews</t>
+          <t>Convlstm Status</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Save the reviewer's verdicts. Rejected frames are left out of the next ConvLSTM retrain.</t>
+          <t>Batch counter of new satellite scans, the deployed ConvLSTM and the result of the last retrain.</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -2194,22 +2194,22 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>/api/frame-review/status</t>
+          <t>/api/retrain/status</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Convlstm Status</t>
+          <t>Deployed models, pending retrains and the retrain history of both models</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Batch counter of new satellite scans, the deployed ConvLSTM and the result of the last retrain.</t>
+          <t>Deployed versions, what is pending and the retrain history of the LSTM and the ConvLSTM.</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>frame-review</t>
+          <t>retrain</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2226,17 +2226,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>/api/retrain/status</t>
+          <t>/api/retrain/runs/{run_id}/curves</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Deployed models, pending retrains and the retrain history of both models</t>
+          <t>Per-epoch learning curves of one retrain run</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Deployed versions, what is pending and the retrain history of the LSTM and the ConvLSTM.</t>
+          <t>Learning curves of one retrain run: training loss, validation metric and learning rate per epoch.</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2258,57 +2258,25 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>/api/retrain/runs/{run_id}/curves</t>
+          <t>/health</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Per-epoch learning curves of one retrain run</t>
+          <t>Health Check</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Learning curves of one retrain run: training loss, validation metric and learning rate per epoch.</t>
+          <t>ตรวจสอบว่า API server ทำงานปกติ</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>retrain</t>
+          <t>system</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>GET</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>/health</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>Health Check</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>ตรวจสอบว่า API server ทำงานปกติ</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>system</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>